<commit_message>
Estado del arte avance 2
</commit_message>
<xml_diff>
--- a/CORRECCIONES TESIS AGOSTO 2026/ESTADO DEL ARTE DESGLOSE.xlsx
+++ b/CORRECCIONES TESIS AGOSTO 2026/ESTADO DEL ARTE DESGLOSE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angel\Desktop\GNLPDA\CORRECCIONES TESIS AGOSTO 2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angeal\Desktop\GNLPDA\CORRECCIONES TESIS AGOSTO 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3C62E13-8D64-4B2D-823B-AA6683FA6B6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD0751C2-F6FA-44F7-958F-A580B38D0F95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{2C1CE7D9-CE8A-41A5-8B84-773C64C88954}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="77040" windowHeight="21120" activeTab="1" xr2:uid="{2C1CE7D9-CE8A-41A5-8B84-773C64C88954}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="97">
   <si>
     <t>Método</t>
   </si>
@@ -180,9 +180,6 @@
 mal condicionadas</t>
   </si>
   <si>
-    <t>Sección</t>
-  </si>
-  <si>
     <t>Regularized LDA</t>
   </si>
   <si>
@@ -304,9 +301,6 @@
   <si>
     <t>Mejorar la eficiencia y robustez de
  NSGA-II para seleccionar subconjuntos de caracteristicas</t>
-  </si>
-  <si>
-    <t>PENDIENTE</t>
   </si>
   <si>
     <t>Reducir el espacio 
@@ -362,13 +356,22 @@
   <si>
     <t>Sí, mediante una 
 transformación intermedia</t>
+  </si>
+  <si>
+    <t>juntar en GA</t>
+  </si>
+  <si>
+    <t>Checar aquí bien las referencias</t>
+  </si>
+  <si>
+    <t>*</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -378,14 +381,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -414,7 +409,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -448,11 +443,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -462,9 +470,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -476,20 +481,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -826,9 +843,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EABEBF3-A5AF-4D6C-8755-961C1765DDC2}">
   <dimension ref="B3:G12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="3" spans="2:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
@@ -848,7 +865,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
         <v>6</v>
       </c>
@@ -868,7 +885,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
         <v>11</v>
       </c>
@@ -888,7 +905,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
         <v>14</v>
       </c>
@@ -908,7 +925,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
         <v>16</v>
       </c>
@@ -928,7 +945,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
         <v>19</v>
       </c>
@@ -948,7 +965,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="2:7" ht="72" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:7" ht="75" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
         <v>20</v>
       </c>
@@ -968,7 +985,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="2:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
         <v>23</v>
       </c>
@@ -988,7 +1005,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="2:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:7" ht="45" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
         <v>27</v>
       </c>
@@ -1008,7 +1025,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
         <v>29</v>
       </c>
@@ -1036,518 +1053,522 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC1CAB86-B352-4717-B4E0-3962B8B36843}">
   <dimension ref="A1:J21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="29.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="52.2" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:10" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="E1" s="12" t="s">
+      <c r="B2" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H5" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="90" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="F1" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="G1" s="12" t="s">
+      <c r="F8" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="105" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="105" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A12" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="105" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="G13" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="H1" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="I1" s="12" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="G2" s="6" t="s">
+      <c r="H13" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A14" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="G14" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="H2" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="I2" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="I3" s="6" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="I4" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H5" s="4" t="s">
+      <c r="H14" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="I14" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="J14" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="E15" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J15" t="s">
         <v>95</v>
       </c>
-      <c r="I5" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="72" x14ac:dyDescent="0.3">
-      <c r="A9" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="G9" s="6" t="s">
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G16" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="H9" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="72" x14ac:dyDescent="0.3">
-      <c r="A10" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="I11" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A13" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="H13" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="I13" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A14" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D14" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="E14" t="s">
-        <v>88</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="G14" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="I14" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="J14" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A15" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="E15" t="s">
-        <v>88</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="H15" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="I15" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="G16" t="s">
-        <v>94</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="I16" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
+      <c r="H16" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="4"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+      <c r="I20" s="4"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>